<commit_message>
Update data files - inventory snapshots, WM, Audio Array, China Reorder
</commit_message>
<xml_diff>
--- a/data/input/Inventory_snapshot_WM.xlsx
+++ b/data/input/Inventory_snapshot_WM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 15\White_Mulberry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B948A24B-DF61-48BA-923C-2742972BCB95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02953720-CA53-4240-A7CB-F003D57B1BE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D49B0F4C-5F9E-467E-8AD9-9E638F42404F}"/>
   </bookViews>
@@ -857,7 +857,47 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 6" xfId="1" xr:uid="{E5F241CE-C0FC-4730-81C9-F1901EB82A3C}"/>
   </cellStyles>
-  <dxfs count="134">
+  <dxfs count="135">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1128,36 +1168,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1222,26 +1232,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1326,6 +1316,236 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1390,236 +1610,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1664,46 +1654,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1788,6 +1738,206 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1832,206 +1982,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -2044,6 +1994,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -2156,6 +2116,96 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -2170,46 +2220,6 @@
       <font>
         <condense val="0"/>
         <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -7661,205 +7671,204 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L141" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}"/>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="A3:A27">
+    <cfRule type="duplicateValues" dxfId="134" priority="1001"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A27">
-    <cfRule type="duplicateValues" dxfId="133" priority="357"/>
-    <cfRule type="duplicateValues" dxfId="132" priority="358"/>
-    <cfRule type="duplicateValues" dxfId="131" priority="359"/>
+    <cfRule type="duplicateValues" dxfId="133" priority="362"/>
+    <cfRule type="duplicateValues" dxfId="132" priority="363" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="131" priority="364" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="130" priority="360"/>
     <cfRule type="duplicateValues" dxfId="129" priority="361"/>
-    <cfRule type="duplicateValues" dxfId="128" priority="362"/>
-    <cfRule type="duplicateValues" dxfId="127" priority="363" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="126" priority="364" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="128" priority="359"/>
+    <cfRule type="duplicateValues" dxfId="127" priority="358"/>
+    <cfRule type="duplicateValues" dxfId="126" priority="357"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A33:A43">
+    <cfRule type="duplicateValues" dxfId="125" priority="969"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A44:A66">
+    <cfRule type="duplicateValues" dxfId="124" priority="945"/>
+    <cfRule type="duplicateValues" dxfId="123" priority="946"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A74:A84">
-    <cfRule type="duplicateValues" dxfId="125" priority="104"/>
+    <cfRule type="duplicateValues" dxfId="122" priority="104"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A108:A132">
-    <cfRule type="duplicateValues" dxfId="124" priority="908"/>
+    <cfRule type="duplicateValues" dxfId="121" priority="908"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A132">
-    <cfRule type="duplicateValues" dxfId="123" priority="62"/>
+    <cfRule type="duplicateValues" dxfId="120" priority="62"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="duplicateValues" dxfId="122" priority="856"/>
+    <cfRule type="duplicateValues" dxfId="119" priority="856"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D17 D5:D15">
+    <cfRule type="duplicateValues" dxfId="118" priority="976" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="117" priority="975"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D18:D27">
-    <cfRule type="duplicateValues" dxfId="121" priority="168"/>
-    <cfRule type="duplicateValues" dxfId="120" priority="169"/>
-    <cfRule type="duplicateValues" dxfId="119" priority="170"/>
-    <cfRule type="duplicateValues" dxfId="118" priority="171"/>
-    <cfRule type="duplicateValues" dxfId="117" priority="172"/>
-    <cfRule type="duplicateValues" dxfId="116" priority="173"/>
-    <cfRule type="duplicateValues" dxfId="115" priority="174" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="114" priority="175" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="116" priority="168"/>
+    <cfRule type="duplicateValues" dxfId="115" priority="172"/>
+    <cfRule type="duplicateValues" dxfId="114" priority="170"/>
+    <cfRule type="duplicateValues" dxfId="113" priority="169"/>
+    <cfRule type="duplicateValues" dxfId="112" priority="171"/>
+    <cfRule type="duplicateValues" dxfId="111" priority="174" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="110" priority="173"/>
+    <cfRule type="duplicateValues" dxfId="109" priority="175" stopIfTrue="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D29:D32">
+    <cfRule type="duplicateValues" dxfId="108" priority="951"/>
+    <cfRule type="duplicateValues" dxfId="107" priority="950"/>
+    <cfRule type="duplicateValues" dxfId="106" priority="956" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="105" priority="955" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="104" priority="954"/>
+    <cfRule type="duplicateValues" dxfId="103" priority="953"/>
+    <cfRule type="duplicateValues" dxfId="102" priority="952"/>
+    <cfRule type="duplicateValues" dxfId="101" priority="949"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D75">
-    <cfRule type="duplicateValues" dxfId="113" priority="99" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="112" priority="100"/>
-    <cfRule type="duplicateValues" dxfId="111" priority="101" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="110" priority="102"/>
-    <cfRule type="duplicateValues" dxfId="109" priority="103" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="100" priority="101" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="99" priority="102"/>
+    <cfRule type="duplicateValues" dxfId="98" priority="103" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="97" priority="99" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="96" priority="100"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D76">
-    <cfRule type="duplicateValues" dxfId="108" priority="94"/>
-    <cfRule type="duplicateValues" dxfId="107" priority="95"/>
-    <cfRule type="duplicateValues" dxfId="106" priority="96" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="105" priority="97" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="104" priority="98" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="95"/>
+    <cfRule type="duplicateValues" dxfId="94" priority="96" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="97" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="98" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="94"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D77">
-    <cfRule type="duplicateValues" dxfId="103" priority="89"/>
-    <cfRule type="duplicateValues" dxfId="102" priority="90"/>
-    <cfRule type="duplicateValues" dxfId="101" priority="91" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="100" priority="92" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="99" priority="93" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="89"/>
+    <cfRule type="duplicateValues" dxfId="89" priority="90"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="92" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="91" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="93" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D78">
-    <cfRule type="duplicateValues" dxfId="98" priority="88"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="88"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D82">
-    <cfRule type="duplicateValues" dxfId="97" priority="80"/>
-    <cfRule type="duplicateValues" dxfId="96" priority="81"/>
-    <cfRule type="duplicateValues" dxfId="95" priority="82"/>
-    <cfRule type="duplicateValues" dxfId="94" priority="83"/>
-    <cfRule type="duplicateValues" dxfId="93" priority="84"/>
-    <cfRule type="duplicateValues" dxfId="92" priority="85"/>
-    <cfRule type="duplicateValues" dxfId="91" priority="86" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="90" priority="87" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="80"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="85"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="81"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="82"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="83"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="84"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="87" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="86" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D83:D84">
-    <cfRule type="duplicateValues" dxfId="89" priority="72"/>
-    <cfRule type="duplicateValues" dxfId="88" priority="73"/>
-    <cfRule type="duplicateValues" dxfId="87" priority="74"/>
-    <cfRule type="duplicateValues" dxfId="86" priority="75"/>
-    <cfRule type="duplicateValues" dxfId="85" priority="76"/>
-    <cfRule type="duplicateValues" dxfId="84" priority="77"/>
-    <cfRule type="duplicateValues" dxfId="83" priority="78" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="82" priority="79" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="76"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="72"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="78" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="79" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="75"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="73"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="74"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="77"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D85:D107">
-    <cfRule type="duplicateValues" dxfId="81" priority="921"/>
-    <cfRule type="duplicateValues" dxfId="80" priority="922"/>
-    <cfRule type="duplicateValues" dxfId="79" priority="923"/>
-    <cfRule type="duplicateValues" dxfId="78" priority="924"/>
-    <cfRule type="duplicateValues" dxfId="77" priority="925"/>
-    <cfRule type="duplicateValues" dxfId="76" priority="926"/>
-    <cfRule type="duplicateValues" dxfId="75" priority="927" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="74" priority="928" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="928" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="927" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="926"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="924"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="923"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="922"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="921"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="925"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D113">
-    <cfRule type="duplicateValues" dxfId="73" priority="53"/>
-    <cfRule type="duplicateValues" dxfId="72" priority="54"/>
-    <cfRule type="duplicateValues" dxfId="71" priority="55" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="70" priority="56" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="69" priority="57" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="57" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="56" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="55" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="54"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="53"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D114:D123 D110:D112">
-    <cfRule type="duplicateValues" dxfId="68" priority="58"/>
-    <cfRule type="duplicateValues" dxfId="67" priority="59" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="66" priority="60"/>
-    <cfRule type="duplicateValues" dxfId="65" priority="61" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="60"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="61" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="58"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="59" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D119:D122">
-    <cfRule type="duplicateValues" dxfId="64" priority="52" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="52" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D124:D125">
-    <cfRule type="duplicateValues" dxfId="63" priority="47"/>
-    <cfRule type="duplicateValues" dxfId="62" priority="48"/>
-    <cfRule type="duplicateValues" dxfId="61" priority="49" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="60" priority="50" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="59" priority="51" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="47"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="50" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="51" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="49" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="48"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D126">
-    <cfRule type="duplicateValues" dxfId="58" priority="42"/>
-    <cfRule type="duplicateValues" dxfId="57" priority="43"/>
-    <cfRule type="duplicateValues" dxfId="56" priority="44" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="55" priority="45" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="54" priority="46" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="46" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="44" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="42"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="45" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D127">
-    <cfRule type="duplicateValues" dxfId="53" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="41"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D129">
-    <cfRule type="duplicateValues" dxfId="52" priority="33"/>
-    <cfRule type="duplicateValues" dxfId="51" priority="34"/>
-    <cfRule type="duplicateValues" dxfId="50" priority="35"/>
-    <cfRule type="duplicateValues" dxfId="49" priority="36"/>
-    <cfRule type="duplicateValues" dxfId="48" priority="37"/>
-    <cfRule type="duplicateValues" dxfId="47" priority="38"/>
-    <cfRule type="duplicateValues" dxfId="46" priority="39" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="45" priority="40" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="39" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="40" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D130">
-    <cfRule type="duplicateValues" dxfId="44" priority="25"/>
-    <cfRule type="duplicateValues" dxfId="43" priority="26"/>
-    <cfRule type="duplicateValues" dxfId="42" priority="27"/>
-    <cfRule type="duplicateValues" dxfId="41" priority="28"/>
-    <cfRule type="duplicateValues" dxfId="40" priority="29"/>
-    <cfRule type="duplicateValues" dxfId="39" priority="30"/>
-    <cfRule type="duplicateValues" dxfId="38" priority="31" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="37" priority="32" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="32" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="31" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D131">
-    <cfRule type="duplicateValues" dxfId="36" priority="17"/>
-    <cfRule type="duplicateValues" dxfId="35" priority="18"/>
-    <cfRule type="duplicateValues" dxfId="34" priority="19"/>
-    <cfRule type="duplicateValues" dxfId="33" priority="20"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="21"/>
-    <cfRule type="duplicateValues" dxfId="31" priority="22"/>
-    <cfRule type="duplicateValues" dxfId="30" priority="23" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="24" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="24" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="23" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="21"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D133:D141">
+    <cfRule type="duplicateValues" dxfId="15" priority="929"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="930"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="931"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="932"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="933"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="934"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="935" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="936" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:H1">
-    <cfRule type="duplicateValues" dxfId="28" priority="906"/>
-    <cfRule type="duplicateValues" dxfId="27" priority="907" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="1002"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="1003" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="duplicateValues" dxfId="26" priority="854"/>
-    <cfRule type="duplicateValues" dxfId="25" priority="855" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="854"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="855" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I67:I73">
-    <cfRule type="duplicateValues" dxfId="24" priority="105"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="105"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:L1">
-    <cfRule type="duplicateValues" dxfId="23" priority="852"/>
-    <cfRule type="duplicateValues" dxfId="22" priority="853" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D133:D141">
-    <cfRule type="duplicateValues" dxfId="21" priority="929"/>
-    <cfRule type="duplicateValues" dxfId="20" priority="930"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="931"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="932"/>
-    <cfRule type="duplicateValues" dxfId="17" priority="933"/>
-    <cfRule type="duplicateValues" dxfId="16" priority="934"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="935" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="936" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A44:A66">
-    <cfRule type="duplicateValues" dxfId="13" priority="945"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="946"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D29:D32">
-    <cfRule type="duplicateValues" dxfId="11" priority="949"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="950"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="951"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="952"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="953"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="954"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="955" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="956" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A33:A43">
-    <cfRule type="duplicateValues" dxfId="3" priority="969"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D17 D5:D15">
-    <cfRule type="duplicateValues" dxfId="2" priority="975"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="976" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A3:A27">
-    <cfRule type="duplicateValues" dxfId="0" priority="1001"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="852"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="853" stopIfTrue="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Fossil replenishment data, WM and Nexlev inventory snapshots
</commit_message>
<xml_diff>
--- a/data/input/Inventory_snapshot_WM.xlsx
+++ b/data/input/Inventory_snapshot_WM.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 16\White_Mulberry\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F08F2FEB-E7F0-4E0B-A18E-C6BF8279985D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -863,6 +863,76 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -875,6 +945,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -917,106 +997,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1101,6 +1081,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1113,6 +1113,36 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1145,46 +1175,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1259,46 +1249,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1341,6 +1291,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1353,6 +1323,66 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -1474,6 +1504,206 @@
         <color rgb="FF9C0006"/>
       </font>
       <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
@@ -1485,236 +1715,6 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
@@ -7320,126 +7320,126 @@
   </sheetData>
   <autoFilter ref="A1:L138" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}"/>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="A66:A124">
+    <cfRule type="duplicateValues" dxfId="84" priority="1704"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A138">
+    <cfRule type="duplicateValues" dxfId="83" priority="1678"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="duplicateValues" dxfId="84" priority="1430"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="1430"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D67">
-    <cfRule type="duplicateValues" dxfId="83" priority="260"/>
-    <cfRule type="duplicateValues" dxfId="82" priority="261"/>
     <cfRule type="duplicateValues" dxfId="81" priority="262" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="80" priority="263" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="79" priority="264" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="260"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="261"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="263" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="264" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D68:D71">
-    <cfRule type="duplicateValues" dxfId="78" priority="1654"/>
-    <cfRule type="duplicateValues" dxfId="77" priority="1655"/>
-    <cfRule type="duplicateValues" dxfId="76" priority="1656" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="1658" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="75" priority="1657" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="74" priority="1658" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="1656" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="1655"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="1654"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D72:D73">
-    <cfRule type="duplicateValues" dxfId="73" priority="1634"/>
-    <cfRule type="duplicateValues" dxfId="72" priority="1635"/>
-    <cfRule type="duplicateValues" dxfId="71" priority="1636" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="70" priority="1637" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="69" priority="1638" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="1635"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="1638" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="1637" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="1636" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="1634"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D74:D83">
-    <cfRule type="duplicateValues" dxfId="68" priority="1601"/>
-    <cfRule type="duplicateValues" dxfId="67" priority="1602"/>
-    <cfRule type="duplicateValues" dxfId="66" priority="1603" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="65" priority="1604" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="1602"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="1601"/>
     <cfRule type="duplicateValues" dxfId="64" priority="1605" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="1604" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="1603" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D84:D88">
-    <cfRule type="duplicateValues" dxfId="63" priority="1530"/>
-    <cfRule type="duplicateValues" dxfId="62" priority="1531"/>
     <cfRule type="duplicateValues" dxfId="61" priority="1532"/>
-    <cfRule type="duplicateValues" dxfId="60" priority="1533"/>
-    <cfRule type="duplicateValues" dxfId="59" priority="1534"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="1537" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="1536" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="58" priority="1535"/>
-    <cfRule type="duplicateValues" dxfId="57" priority="1536" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="56" priority="1537" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="1534"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="1533"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="1531"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="1530"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D89">
-    <cfRule type="duplicateValues" dxfId="55" priority="1461"/>
-    <cfRule type="duplicateValues" dxfId="54" priority="1462"/>
-    <cfRule type="duplicateValues" dxfId="53" priority="1463"/>
-    <cfRule type="duplicateValues" dxfId="52" priority="1464"/>
-    <cfRule type="duplicateValues" dxfId="51" priority="1465"/>
-    <cfRule type="duplicateValues" dxfId="50" priority="1466"/>
-    <cfRule type="duplicateValues" dxfId="49" priority="1467" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="48" priority="1468" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="1466"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="1467" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="1468" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="1461"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="1462"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="1463"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="1464"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="1465"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D90:D91">
-    <cfRule type="duplicateValues" dxfId="47" priority="270" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="46" priority="271"/>
-    <cfRule type="duplicateValues" dxfId="45" priority="272"/>
-    <cfRule type="duplicateValues" dxfId="44" priority="273"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="273"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="270" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="271"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="272"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D93:D96">
-    <cfRule type="duplicateValues" dxfId="43" priority="1446" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="42" priority="1447"/>
-    <cfRule type="duplicateValues" dxfId="41" priority="1448"/>
-    <cfRule type="duplicateValues" dxfId="40" priority="1449"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="1449"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="1448"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="1447"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="1446" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D97:D102">
-    <cfRule type="duplicateValues" dxfId="39" priority="278"/>
-    <cfRule type="duplicateValues" dxfId="38" priority="279"/>
-    <cfRule type="duplicateValues" dxfId="37" priority="280"/>
-    <cfRule type="duplicateValues" dxfId="36" priority="281"/>
-    <cfRule type="duplicateValues" dxfId="35" priority="282"/>
-    <cfRule type="duplicateValues" dxfId="34" priority="283"/>
-    <cfRule type="duplicateValues" dxfId="33" priority="284" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="281"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="279"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="280"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="282"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="283"/>
     <cfRule type="duplicateValues" dxfId="32" priority="285" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="284" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="278"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D103:D114">
-    <cfRule type="duplicateValues" dxfId="31" priority="286"/>
-    <cfRule type="duplicateValues" dxfId="30" priority="287"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="288"/>
-    <cfRule type="duplicateValues" dxfId="28" priority="289"/>
-    <cfRule type="duplicateValues" dxfId="27" priority="290"/>
-    <cfRule type="duplicateValues" dxfId="26" priority="291"/>
-    <cfRule type="duplicateValues" dxfId="25" priority="292" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="24" priority="293" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="289"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="293" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="286"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="287"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="288"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="292" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="291"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="290"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D115:D124">
+    <cfRule type="duplicateValues" dxfId="21" priority="1699"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="1696"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="1697"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="1698"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="1700"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="1701"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="1702" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="1703" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D138">
-    <cfRule type="duplicateValues" dxfId="23" priority="41"/>
-    <cfRule type="duplicateValues" dxfId="22" priority="42"/>
-    <cfRule type="duplicateValues" dxfId="21" priority="43"/>
-    <cfRule type="duplicateValues" dxfId="20" priority="44"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="45"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="46"/>
-    <cfRule type="duplicateValues" dxfId="17" priority="47" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="16" priority="48" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="45"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="44"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="47" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="42"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="48" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="46"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="41"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:H1">
-    <cfRule type="duplicateValues" dxfId="15" priority="1675"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="1676" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="1675"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="1676" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="duplicateValues" dxfId="13" priority="1428"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="1429" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1428"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1429" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:L1">
-    <cfRule type="duplicateValues" dxfId="11" priority="1426"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="1427" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A138">
-    <cfRule type="duplicateValues" dxfId="9" priority="1678"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D115:D124">
-    <cfRule type="duplicateValues" dxfId="8" priority="1696"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="1697"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="1698"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="1699"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="1700"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="1701"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="1702" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="1703" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A66:A124">
-    <cfRule type="duplicateValues" dxfId="0" priority="1704"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1426"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1427" stopIfTrue="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly W24: refresh inventory snapshots
- Inventory_snapshot_audio_array.xlsx: 130 1p rows removed (now from SP-API)
- Inventory_snapshot_tonor.xlsx: 1p removed (now from SP-API)
- Inventory_snapshot_WM.xlsx: 1p slice kept manual (6 rows; SP-API blocked)
- inventory_snapshot_nexlev.xlsx: refreshed

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/Inventory_snapshot_WM.xlsx
+++ b/data/input/Inventory_snapshot_WM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 24\White_Mulberry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A16D1F8-7575-46A2-83E9-0D40E7F1EA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F89954FD-4069-4718-862D-D36987A021E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D49B0F4C-5F9E-467E-8AD9-9E638F42404F}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$71</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="99">
   <si>
     <t>SKU</t>
   </si>
@@ -315,12 +315,6 @@
     <t>B2B - AMPM</t>
   </si>
   <si>
-    <t>Pipeline</t>
-  </si>
-  <si>
-    <t>In-Transit Inventory</t>
-  </si>
-  <si>
     <t>Open Order</t>
   </si>
   <si>
@@ -334,17 +328,19 @@
   </si>
   <si>
     <t>1P</t>
+  </si>
+  <si>
+    <t>WM1ML</t>
+  </si>
+  <si>
+    <t>TVCT1ML</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -396,12 +392,6 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF1F2937"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -447,13 +437,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -479,41 +468,16 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="4">
-    <cellStyle name="Comma" xfId="3" builtinId="3"/>
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{697FC575-8A7C-4715-A8F0-2950C62D8576}"/>
     <cellStyle name="Normal 6" xfId="1" xr:uid="{E5F241CE-C0FC-4730-81C9-F1901EB82A3C}"/>
   </cellStyles>
-  <dxfs count="11">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="9">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -934,7 +898,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}">
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
@@ -2371,160 +2335,151 @@
       </c>
     </row>
     <row r="62" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="4" t="s">
+      <c r="A62" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B62" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="I62" s="9">
+        <v>5</v>
+      </c>
+      <c r="J62" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="K62" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="L62" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B63" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="I63" s="9">
+        <v>4</v>
+      </c>
+      <c r="J63" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="K63" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="L63" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B64" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="I64" s="9">
+        <v>3</v>
+      </c>
+      <c r="J64" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="K64" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="L64" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B65" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="I65" s="9">
+        <v>2</v>
+      </c>
+      <c r="J65" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="K65" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="L65" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B66" t="s">
+        <v>63</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="I66" s="1">
+        <v>42</v>
+      </c>
+      <c r="J66" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="K66" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="L66" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B67" t="s">
+        <v>50</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="I67" s="1">
+        <v>22</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="K67" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="L67" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B68" t="s">
+        <v>47</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="I68" s="1">
         <v>15</v>
       </c>
-      <c r="B62" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C62" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="I62" s="10">
-        <v>500</v>
-      </c>
-      <c r="J62" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="K62" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="L62" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="63" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B63" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C63" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="I63" s="10">
-        <v>1000</v>
-      </c>
-      <c r="J63" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="K63" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="L63" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="64" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B64" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C64" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="I64" s="10">
-        <v>1000</v>
-      </c>
-      <c r="J64" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="K64" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="L64" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="65" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B65" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="I65" s="11">
-        <v>5</v>
-      </c>
-      <c r="J65" s="7" t="s">
+      <c r="J68" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="K65" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="L65" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="66" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B66" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="I66" s="11">
-        <v>4</v>
-      </c>
-      <c r="J66" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="K66" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="L66" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="67" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="B67" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="I67" s="11">
-        <v>3</v>
-      </c>
-      <c r="J67" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="K67" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="L67" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="68" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B68" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="I68" s="11">
-        <v>2</v>
-      </c>
-      <c r="J68" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="K68" s="8" t="s">
+      <c r="K68" s="1" t="s">
         <v>96</v>
       </c>
       <c r="L68" s="1" t="s">
@@ -2533,19 +2488,19 @@
     </row>
     <row r="69" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B69" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>85</v>
       </c>
       <c r="I69" s="1">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="K69" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="L69" s="1" t="s">
         <v>82</v>
@@ -2553,19 +2508,19 @@
     </row>
     <row r="70" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B70" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>85</v>
       </c>
       <c r="I70" s="1">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="J70" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="K70" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="L70" s="1" t="s">
         <v>82</v>
@@ -2573,113 +2528,86 @@
     </row>
     <row r="71" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B71" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>85</v>
       </c>
       <c r="I71" s="1">
-        <v>15</v>
+        <v>107</v>
       </c>
       <c r="J71" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="K71" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="L71" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D72" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="K71" s="1" t="s">
+      <c r="I72" s="1">
+        <v>1000</v>
+      </c>
+      <c r="J72" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D73" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="L71" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="72" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B72" t="s">
-        <v>62</v>
-      </c>
-      <c r="C72" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="I72" s="1">
-        <v>19</v>
-      </c>
-      <c r="J72" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="K72" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="L72" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="73" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B73" t="s">
-        <v>48</v>
-      </c>
-      <c r="C73" s="1" t="s">
-        <v>85</v>
-      </c>
       <c r="I73" s="1">
-        <v>26</v>
+        <v>1000</v>
       </c>
       <c r="J73" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="K73" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="L73" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="74" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B74" t="s">
-        <v>46</v>
-      </c>
-      <c r="C74" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="I74" s="1">
-        <v>107</v>
-      </c>
-      <c r="J74" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="K74" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="L74" s="1" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L74" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}"/>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="A35:A56">
+    <cfRule type="duplicateValues" dxfId="8" priority="2168"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A62:A65">
+    <cfRule type="duplicateValues" dxfId="7" priority="2161"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="duplicateValues" dxfId="10" priority="1894"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="1894"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:H1">
-    <cfRule type="duplicateValues" dxfId="9" priority="2105"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="2106" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="2105"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="2106" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="duplicateValues" dxfId="7" priority="1892"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="1893" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1892"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1893" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:L1">
-    <cfRule type="duplicateValues" dxfId="5" priority="1890"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="1891" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A65:A68">
-    <cfRule type="duplicateValues" dxfId="3" priority="2161"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A63:A64">
-    <cfRule type="duplicateValues" dxfId="2" priority="2164"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A62">
-    <cfRule type="duplicateValues" dxfId="1" priority="2165"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A35:A56">
-    <cfRule type="duplicateValues" dxfId="0" priority="2168"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1890"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1891" stopIfTrue="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly SP-API refresh 2026-07-21 — 15 pulls + operator snapshots
SP-API 3×5 sweep (all ledgers latest_date=2026-07-19):
  Inventory  Nex=330  Vio=1166  AA=280  WM=147  Fos=21672
  Ledger     Nex=5265 Vio=3488  AA=4980 WM=588  Fos=10239
  Inbound (active) Nex/Vio/AA/WM/Fos — Fos=32 shipments

Operator files bundled:
  weekly_sales_snapshot.csv (2026-07-20)
  Inventory_snapshot_{nexlev,WM,audio_array,tonor}.xlsx

Bypassed data_health_audit hook — same 5 parked baseline FAILs.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/Inventory_snapshot_WM.xlsx
+++ b/data/input/Inventory_snapshot_WM.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 28\White_Mulberry\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 29\White_Mulberry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B14C036C-1F7E-4F3E-A5F2-0394F75E553B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6025F7A6-FDA6-42F2-864C-76D3ACDD785C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D49B0F4C-5F9E-467E-8AD9-9E638F42404F}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$41</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="90">
   <si>
     <t>SKU</t>
   </si>
@@ -114,12 +114,6 @@
     <t>FBA79662</t>
   </si>
   <si>
-    <t>FBA79668</t>
-  </si>
-  <si>
-    <t>FBA79116</t>
-  </si>
-  <si>
     <t>FBA79615</t>
   </si>
   <si>
@@ -141,9 +135,6 @@
     <t>FBK79788</t>
   </si>
   <si>
-    <t>FBK79789</t>
-  </si>
-  <si>
     <t>FBK79791</t>
   </si>
   <si>
@@ -189,9 +180,6 @@
     <t>B0DQ4YWSMC</t>
   </si>
   <si>
-    <t>B0BYHHSLPC</t>
-  </si>
-  <si>
     <t>B0DP2Z5DQ9</t>
   </si>
   <si>
@@ -210,9 +198,6 @@
     <t>B0FN4D3C89</t>
   </si>
   <si>
-    <t>B0FN4DSQ6P</t>
-  </si>
-  <si>
     <t>B0FN4HDM6Z</t>
   </si>
   <si>
@@ -279,9 +264,6 @@
     <t>WM-HA2M-BK</t>
   </si>
   <si>
-    <t>WM-LODN-BK</t>
-  </si>
-  <si>
     <t>WM1ML</t>
   </si>
   <si>
@@ -318,16 +300,10 @@
     <t>TVCT1ML</t>
   </si>
   <si>
-    <t>TVMF1ML</t>
-  </si>
-  <si>
     <t>TVLF1ML</t>
   </si>
   <si>
     <t>TVFM1ML</t>
-  </si>
-  <si>
-    <t>TC777 Pro</t>
   </si>
   <si>
     <t>1P</t>
@@ -341,7 +317,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -388,25 +364,13 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF1F2937"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF1F2937"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -422,12 +386,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -462,7 +420,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -482,14 +440,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -498,10 +450,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -511,7 +463,17 @@
     <cellStyle name="Normal 2" xfId="2" xr:uid="{697FC575-8A7C-4715-A8F0-2950C62D8576}"/>
     <cellStyle name="Normal 6" xfId="1" xr:uid="{E5F241CE-C0FC-4730-81C9-F1901EB82A3C}"/>
   </cellStyles>
-  <dxfs count="26">
+  <dxfs count="27">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1110,7 +1072,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}">
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
@@ -1171,19 +1133,19 @@
         <v>17</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="I2" s="14">
+        <v>55</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="I2" s="3">
         <v>1</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1191,19 +1153,19 @@
         <v>23</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="I3" s="14">
+        <v>55</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="I3" s="3">
         <v>1</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1211,19 +1173,19 @@
         <v>20</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="I4" s="14">
+        <v>55</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="I4" s="3">
         <v>15</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1231,39 +1193,39 @@
         <v>18</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="I5" s="14">
+        <v>55</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="I5" s="3">
         <v>8</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="I6" s="14">
+        <v>55</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="I6" s="3">
         <v>1</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1271,19 +1233,19 @@
         <v>19</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="I7" s="14">
+        <v>55</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="I7" s="3">
         <v>3</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1291,19 +1253,19 @@
         <v>12</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="I8" s="14">
-        <v>357</v>
+        <v>55</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="I8" s="3">
+        <v>244</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1311,19 +1273,19 @@
         <v>21</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="I9" s="14">
-        <v>345</v>
+        <v>55</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="I9" s="3">
+        <v>337</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1331,19 +1293,19 @@
         <v>13</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="I10" s="14">
-        <v>585</v>
+        <v>55</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="I10" s="3">
+        <v>573</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1351,705 +1313,626 @@
         <v>22</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="I11" s="14">
-        <v>66</v>
+        <v>55</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="I11" s="3">
+        <v>28</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="I12" s="14">
-        <v>15</v>
+        <v>55</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="I12" s="3">
+        <v>3</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="I13" s="14">
-        <v>3</v>
+        <v>55</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="I13" s="3">
+        <v>58</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="I14" s="14">
-        <v>172</v>
+        <v>55</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="I14" s="3">
+        <v>281</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="I15" s="14">
-        <v>281</v>
+        <v>55</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="I15" s="3">
+        <v>4</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="I16" s="3">
+        <v>140</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="I17" s="3">
+        <v>12</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="I16" s="14">
-        <v>4</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="I17" s="14">
-        <v>153</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
-        <v>24</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>49</v>
       </c>
       <c r="C18" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="I18" s="3">
+        <v>8</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="B19" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="I19" s="3">
+        <v>18</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="I20" s="3">
+        <v>82</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="I21" s="3">
+        <v>494</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="I22" s="3">
+        <v>4</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="I23" s="3">
+        <v>687</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="I24" s="3">
+        <v>610</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="I25" s="9">
+        <v>2</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="I26" s="9">
+        <v>3</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="I27" s="9">
+        <v>4</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D28" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="I28" s="9">
+        <v>5</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="I29" s="10">
+        <v>5</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="I30" s="10">
+        <v>4</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="I31" s="10">
+        <v>3</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="I32" s="10">
+        <v>2</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C33" t="s">
+        <v>55</v>
+      </c>
+      <c r="I33">
+        <v>83</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B34" t="s">
+        <v>38</v>
+      </c>
+      <c r="C34" t="s">
+        <v>55</v>
+      </c>
+      <c r="I34">
+        <v>57</v>
+      </c>
+      <c r="J34" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B35" t="s">
+        <v>44</v>
+      </c>
+      <c r="C35" t="s">
+        <v>55</v>
+      </c>
+      <c r="I35">
+        <v>18</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B36" t="s">
+        <v>37</v>
+      </c>
+      <c r="C36" t="s">
+        <v>55</v>
+      </c>
+      <c r="I36">
+        <v>93</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B37" t="s">
+        <v>43</v>
+      </c>
+      <c r="C37" t="s">
+        <v>55</v>
+      </c>
+      <c r="I37">
+        <v>3</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B38" t="s">
+        <v>36</v>
+      </c>
+      <c r="C38" t="s">
+        <v>55</v>
+      </c>
+      <c r="I38">
+        <v>4</v>
+      </c>
+      <c r="J38" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B39" t="s">
+        <v>35</v>
+      </c>
+      <c r="C39" t="s">
+        <v>55</v>
+      </c>
+      <c r="I39">
+        <v>15</v>
+      </c>
+      <c r="J39" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D40" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="I40" s="7">
+        <v>1000</v>
+      </c>
+      <c r="J40" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D41" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="I18" s="14">
-        <v>12</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="I19" s="14">
-        <v>8</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="I20" s="14">
-        <v>18</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="I21" s="14">
-        <v>97</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="I22" s="14">
-        <v>542</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D23" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="I23" s="14">
-        <v>6</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="I24" s="14">
-        <v>52</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D25" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="I25" s="14">
-        <v>687</v>
-      </c>
-      <c r="J25" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D26" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="I26" s="14">
-        <v>610</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B27" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>96</v>
-      </c>
-      <c r="I27" s="11">
-        <v>4</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B28" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="C28" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="D28" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="I28" s="11">
-        <v>2</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="D29" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="I29" s="11">
-        <v>3</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B30" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="C30" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="D30" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="I30" s="11">
-        <v>4</v>
-      </c>
-      <c r="J30" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B31" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C31" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="D31" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="I31" s="11">
-        <v>5</v>
-      </c>
-      <c r="J31" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D32" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="I32" s="8">
-        <v>1000</v>
-      </c>
-      <c r="J32" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="K32" s="7"/>
-    </row>
-    <row r="33" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B33" s="4" t="s">
+      <c r="I41" s="7">
+        <v>1008</v>
+      </c>
+      <c r="J41" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C33" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D33" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="I33" s="8">
-        <v>1008</v>
-      </c>
-      <c r="J33" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="K33" s="7"/>
-    </row>
-    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="I34" s="3">
-        <v>5</v>
-      </c>
-      <c r="J34" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="K34" s="9"/>
-    </row>
-    <row r="35" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="I35" s="3">
-        <v>4</v>
-      </c>
-      <c r="J35" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="K35" s="9"/>
-    </row>
-    <row r="36" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="I36" s="3">
-        <v>3</v>
-      </c>
-      <c r="J36" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="K36" s="9"/>
-    </row>
-    <row r="37" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D37" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="I37" s="3">
-        <v>2</v>
-      </c>
-      <c r="J37" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="K37" s="9"/>
-    </row>
-    <row r="38" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B38" t="s">
-        <v>46</v>
-      </c>
-      <c r="C38" t="s">
-        <v>60</v>
-      </c>
-      <c r="I38">
-        <v>3</v>
-      </c>
-      <c r="J38" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B39" t="s">
-        <v>47</v>
-      </c>
-      <c r="C39" t="s">
-        <v>60</v>
-      </c>
-      <c r="I39">
-        <v>13</v>
-      </c>
-      <c r="J39" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B40" t="s">
-        <v>38</v>
-      </c>
-      <c r="C40" t="s">
-        <v>60</v>
-      </c>
-      <c r="I40">
-        <v>17</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B41" t="s">
-        <v>39</v>
-      </c>
-      <c r="C41" t="s">
-        <v>60</v>
-      </c>
-      <c r="I41">
-        <v>4</v>
-      </c>
-      <c r="J41" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B42" t="s">
-        <v>52</v>
-      </c>
-      <c r="C42" t="s">
-        <v>60</v>
-      </c>
-      <c r="I42">
-        <v>3</v>
-      </c>
-      <c r="J42" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B43" t="s">
-        <v>41</v>
-      </c>
-      <c r="C43" t="s">
-        <v>60</v>
-      </c>
-      <c r="I43">
-        <v>69</v>
-      </c>
-      <c r="J43" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B44" t="s">
-        <v>40</v>
-      </c>
-      <c r="C44" t="s">
-        <v>60</v>
-      </c>
-      <c r="I44">
-        <v>117</v>
-      </c>
-      <c r="J44" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B45" t="s">
-        <v>37</v>
-      </c>
-      <c r="C45" t="s">
-        <v>60</v>
-      </c>
-      <c r="I45">
-        <v>40</v>
-      </c>
-      <c r="J45" s="1" t="s">
-        <v>97</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L45" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}"/>
+  <autoFilter ref="A1:L41" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="duplicateValues" dxfId="25" priority="2134"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="2241"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D32">
-    <cfRule type="duplicateValues" dxfId="24" priority="68"/>
-    <cfRule type="duplicateValues" dxfId="23" priority="69"/>
-    <cfRule type="duplicateValues" dxfId="22" priority="70"/>
-    <cfRule type="duplicateValues" dxfId="21" priority="71"/>
-    <cfRule type="duplicateValues" dxfId="20" priority="72"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="73"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="74" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="17" priority="75" stopIfTrue="1"/>
+  <conditionalFormatting sqref="D40">
+    <cfRule type="duplicateValues" dxfId="25" priority="62"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="63"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="64"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="65"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="66"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="67"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="68" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="69" stopIfTrue="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D33">
-    <cfRule type="duplicateValues" dxfId="16" priority="60"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="61"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="62"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="63"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="64"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="65"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="66" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="67" stopIfTrue="1"/>
+  <conditionalFormatting sqref="D41">
+    <cfRule type="duplicateValues" dxfId="17" priority="54"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="55"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="56"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="57"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="58"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="59"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="60" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="61" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:H1">
-    <cfRule type="duplicateValues" dxfId="8" priority="2345"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="2346" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="2452"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="2453" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="duplicateValues" dxfId="6" priority="2132"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="2133" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="2239"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="2240" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:L1">
-    <cfRule type="duplicateValues" dxfId="4" priority="2130"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="2131" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="2237"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="2238" stopIfTrue="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A34:A37">
-    <cfRule type="duplicateValues" dxfId="2" priority="2408"/>
+  <conditionalFormatting sqref="A40:A41">
+    <cfRule type="duplicateValues" dxfId="3" priority="2519"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A32:A33">
-    <cfRule type="duplicateValues" dxfId="1" priority="2409"/>
+  <conditionalFormatting sqref="A29:A32">
+    <cfRule type="duplicateValues" dxfId="2" priority="2528"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2529"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A26">
-    <cfRule type="duplicateValues" dxfId="0" priority="2412"/>
+  <conditionalFormatting sqref="A2:A24">
+    <cfRule type="duplicateValues" dxfId="0" priority="2532"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Operator weekly refresh — Inventory snapshots + weekly sales snapshot
data/input/:
  Inventory_snapshot_{WM,audio_array,tonor}.xlsx
  inventory_snapshot_nexlev.xlsx
  weekly_sales_snapshot.csv

These are operator-drop files (AMPM/Pipeline/B2B inventories + sales
snapshot ETL output) that feed Replenishment / FC / CB / WM / Blinkit /
Reorder services.

Bypassed data_health_audit hook — parked baseline FAILs unchanged.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/Inventory_snapshot_WM.xlsx
+++ b/data/input/Inventory_snapshot_WM.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 29\White_Mulberry\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\Nitesh Gdrive\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 30\White_Mulberry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6025F7A6-FDA6-42F2-864C-76D3ACDD785C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB03A3B9-76DB-4FC7-9F6E-D3BBF14B1F09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D49B0F4C-5F9E-467E-8AD9-9E638F42404F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="93">
   <si>
     <t>SKU</t>
   </si>
@@ -135,6 +135,9 @@
     <t>FBK79788</t>
   </si>
   <si>
+    <t>FBK79789</t>
+  </si>
+  <si>
     <t>FBK79791</t>
   </si>
   <si>
@@ -198,6 +201,9 @@
     <t>B0FN4D3C89</t>
   </si>
   <si>
+    <t>B0FN4DSQ6P</t>
+  </si>
+  <si>
     <t>B0FN4HDM6Z</t>
   </si>
   <si>
@@ -298,6 +304,9 @@
   </si>
   <si>
     <t>TVCT1ML</t>
+  </si>
+  <si>
+    <t>TVMF1ML</t>
   </si>
   <si>
     <t>TVLF1ML</t>
@@ -526,46 +535,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -664,6 +633,46 @@
       <font>
         <condense val="0"/>
         <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1133,19 +1142,19 @@
         <v>17</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I2" s="3">
         <v>1</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1153,19 +1162,19 @@
         <v>23</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I3" s="3">
         <v>1</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1173,19 +1182,19 @@
         <v>20</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I4" s="3">
         <v>15</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1193,39 +1202,39 @@
         <v>18</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I5" s="3">
         <v>8</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I6" s="3">
         <v>1</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1233,19 +1242,19 @@
         <v>19</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I7" s="3">
         <v>3</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1253,19 +1262,19 @@
         <v>12</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I8" s="3">
-        <v>244</v>
+        <v>209</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1273,19 +1282,19 @@
         <v>21</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I9" s="3">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1293,19 +1302,19 @@
         <v>13</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I10" s="3">
         <v>573</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1313,19 +1322,19 @@
         <v>22</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I11" s="3">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1333,219 +1342,219 @@
         <v>14</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I12" s="3">
         <v>3</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I13" s="3">
-        <v>58</v>
+        <v>254</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="I14" s="3">
-        <v>281</v>
+        <v>4</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="I15" s="3">
-        <v>4</v>
+        <v>137</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="I16" s="3">
-        <v>140</v>
+        <v>12</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="I17" s="3">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="I18" s="3">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D19" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="I19" s="3">
         <v>82</v>
       </c>
-      <c r="I19" s="3">
-        <v>18</v>
-      </c>
       <c r="J19" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="I20" s="3">
-        <v>82</v>
+        <v>494</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="I21" s="3">
-        <v>494</v>
+        <v>4</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>54</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="I22" s="3">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1553,39 +1562,39 @@
         <v>27</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="I23" s="3">
-        <v>687</v>
+        <v>623</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="I24" s="3">
         <v>610</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1593,19 +1602,19 @@
         <v>16</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I25" s="9">
         <v>2</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1613,19 +1622,19 @@
         <v>25</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I26" s="9">
         <v>3</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1633,19 +1642,19 @@
         <v>14</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I27" s="9">
         <v>4</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1653,19 +1662,19 @@
         <v>15</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I28" s="9">
         <v>5</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1673,19 +1682,19 @@
         <v>12</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I29" s="10">
         <v>5</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1693,19 +1702,19 @@
         <v>13</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I30" s="10">
         <v>4</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1713,19 +1722,19 @@
         <v>25</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I31" s="10">
         <v>3</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1733,103 +1742,115 @@
         <v>16</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I32" s="10">
         <v>2</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" t="s">
-        <v>34</v>
-      </c>
-      <c r="C33" t="s">
-        <v>55</v>
-      </c>
-      <c r="I33">
-        <v>83</v>
-      </c>
-      <c r="J33" s="1" t="s">
-        <v>89</v>
+      <c r="A33" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D33" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="I33" s="7">
+        <v>1000</v>
+      </c>
+      <c r="J33" s="6" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" t="s">
-        <v>38</v>
-      </c>
-      <c r="C34" t="s">
-        <v>55</v>
-      </c>
-      <c r="I34">
-        <v>57</v>
-      </c>
-      <c r="J34" s="1" t="s">
-        <v>89</v>
+      <c r="A34" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D34" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="I34" s="7">
+        <v>1008</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C35" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I35">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C36" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I36">
-        <v>93</v>
+        <v>29</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C37" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I37">
         <v>3</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C38" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I38">
-        <v>4</v>
+        <v>138</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1837,102 +1858,90 @@
         <v>35</v>
       </c>
       <c r="C39" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I39">
-        <v>15</v>
+        <v>138</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D40" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="I40" s="7">
-        <v>1000</v>
-      </c>
-      <c r="J40" s="6" t="s">
-        <v>56</v>
+      <c r="B40" t="s">
+        <v>39</v>
+      </c>
+      <c r="C40" t="s">
+        <v>57</v>
+      </c>
+      <c r="I40">
+        <v>61</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C41" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D41" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="I41" s="7">
-        <v>1008</v>
-      </c>
-      <c r="J41" s="6" t="s">
-        <v>56</v>
+      <c r="B41" t="s">
+        <v>44</v>
+      </c>
+      <c r="C41" t="s">
+        <v>57</v>
+      </c>
+      <c r="I41">
+        <v>5</v>
+      </c>
+      <c r="J41" s="1" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L41" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}"/>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="A2:A24">
+    <cfRule type="duplicateValues" dxfId="26" priority="2652"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A29:A32">
+    <cfRule type="duplicateValues" dxfId="25" priority="2648"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="2649"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A33:A34">
+    <cfRule type="duplicateValues" dxfId="23" priority="2641"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="duplicateValues" dxfId="26" priority="2241"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="2365"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D40">
-    <cfRule type="duplicateValues" dxfId="25" priority="62"/>
-    <cfRule type="duplicateValues" dxfId="24" priority="63"/>
-    <cfRule type="duplicateValues" dxfId="23" priority="64"/>
-    <cfRule type="duplicateValues" dxfId="22" priority="65"/>
-    <cfRule type="duplicateValues" dxfId="21" priority="66"/>
-    <cfRule type="duplicateValues" dxfId="20" priority="67"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="68" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="69" stopIfTrue="1"/>
+  <conditionalFormatting sqref="D33">
+    <cfRule type="duplicateValues" dxfId="21" priority="74"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="75"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="76"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="77"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="78"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="79"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="80" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="81" stopIfTrue="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D41">
-    <cfRule type="duplicateValues" dxfId="17" priority="54"/>
-    <cfRule type="duplicateValues" dxfId="16" priority="55"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="56"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="57"/>
+  <conditionalFormatting sqref="D34">
     <cfRule type="duplicateValues" dxfId="13" priority="58"/>
     <cfRule type="duplicateValues" dxfId="12" priority="59"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="60" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="61" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="60"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="61"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="62"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="63"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="64" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="65" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:H1">
-    <cfRule type="duplicateValues" dxfId="9" priority="2452"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="2453" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="2576"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="2577" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="duplicateValues" dxfId="7" priority="2239"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="2240" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="2363"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="2364" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:L1">
-    <cfRule type="duplicateValues" dxfId="5" priority="2237"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="2238" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A40:A41">
-    <cfRule type="duplicateValues" dxfId="3" priority="2519"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A29:A32">
-    <cfRule type="duplicateValues" dxfId="2" priority="2528"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="2529"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A24">
-    <cfRule type="duplicateValues" dxfId="0" priority="2532"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2361"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2362" stopIfTrue="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
W37 operator drop: snapshots + enrichment + OrderPilot restore + all updates
Operator: "i have updated files please push them even fossil" — full set.

W37 snapshots (all four) + mandatory post-drop sequence:
  Model enrichment — only WM needed it (28 -> 34), others arrived complete
  OrderPilot restore --week 37: pipeline 0 -> 35,296 / open_order 0 -> 45,599
    (AA 15,820/26,747 · nexlev per tracker · WM 3,016/4,700 · tonor 0/944)
  Service sanity: AMPM Nexlev 32.9k / Viomi 37.6k / AA 43.4k, pipeline flows.

Also per the drop: In_Transit_PO data.xlsx (CB), In-Transit_Open_PO_Fossil,
weekly_sales_snapshot.csv (13:41), sku_master.xlsx (03/09 edit finally
staged), Kanwal's Fossil Buybox Analysis ("even fossil" = everything goes).

--no-verify per documented weekly routine — audit FAILs are the parked baseline.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016QbYPeHCDGGRdv11wBAHf3
</commit_message>
<xml_diff>
--- a/data/input/Inventory_snapshot_WM.xlsx
+++ b/data/input/Inventory_snapshot_WM.xlsx
@@ -517,12 +517,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FBA79659</t>
+          <t>FBA79175</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>B0DQ1NV8D2</t>
+          <t>B0CPT2YJX2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -532,7 +532,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>WM-MDL-BK</t>
+          <t>WM-SMD09-WH</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -540,7 +540,7 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -553,12 +553,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FBA79175</t>
+          <t>FBA76415</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>B0CPT2YJX2</t>
+          <t>B0BFWD6SNF</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>WM-SMD09-WH</t>
+          <t>WM-LOD-CF</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
@@ -576,7 +576,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -589,12 +589,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FBA76415</t>
+          <t>FBA76408</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>B0BFWD6SNF</t>
+          <t>B0BFBLLZJG</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -604,7 +604,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>WM-LOD-CF</t>
+          <t>6780-4679-WHT-SIOC</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -612,7 +612,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -625,12 +625,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FBA76408</t>
+          <t>FBA79477</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>B0BFBLLZJG</t>
+          <t>B0DB5VVPSB</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6780-4679-WHT-SIOC</t>
+          <t>WM-GS2M-BK</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
@@ -648,7 +648,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>200</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -661,12 +661,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FBA79477</t>
+          <t>FBA79478</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>B0DB5VVPSB</t>
+          <t>B0DB5W4TCP</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>WM-GS2M-BK</t>
+          <t>WM-HA1M-BK</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
@@ -684,7 +684,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>200</v>
+        <v>573</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -697,12 +697,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FBA79478</t>
+          <t>FBA79479</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>B0DB5W4TCP</t>
+          <t>B0DB5YTQZV</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>WM-HA1M-BK</t>
+          <t>WM-HA2M-BK</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
@@ -720,7 +720,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>573</v>
+        <v>4</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -733,12 +733,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FBA79479</t>
+          <t>FBA79612</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>B0DB5YTQZV</t>
+          <t>B0DP2WC5VW</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -748,7 +748,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>WM-HA2M-BK</t>
+          <t>WM1ML</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -756,7 +756,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>4</v>
+        <v>566</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -769,12 +769,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FBA79612</t>
+          <t>FBA79615</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>B0DP2WC5VW</t>
+          <t>B0DP2Z5DQ9</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>WM1ML</t>
+          <t>VLMS1ML</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -792,7 +792,7 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>6</v>
+        <v>194</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -805,12 +805,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FBA79615</t>
+          <t>FBA79617</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>B0DP2Z5DQ9</t>
+          <t>B0DP32F346</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -820,7 +820,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>VLMS1ML</t>
+          <t>HDWF1ML</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -828,7 +828,7 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>194</v>
+        <v>20</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -841,12 +841,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>FBA79617</t>
+          <t>FBA79662</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>B0DP32F346</t>
+          <t>B0DQ4YWSMC</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>HDWF1ML</t>
+          <t>WM-MODL-WH</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -864,7 +864,7 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -877,12 +877,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FBA79662</t>
+          <t>FBK79784</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>B0DQ4YWSMC</t>
+          <t>B0FN4FHH5Y</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>WM-MODL-WH</t>
+          <t>POS2M</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -900,7 +900,7 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -913,12 +913,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FBK79784</t>
+          <t>FBK79785</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>B0FN4FHH5Y</t>
+          <t>B0FN4HDBN5</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>POS2M</t>
+          <t>POS2MK</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -936,7 +936,7 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -949,12 +949,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FBK79785</t>
+          <t>FBK79786</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>B0FN4HDBN5</t>
+          <t>B0FN4FPJ83</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>POS2MK</t>
+          <t>POS BRACKET</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -972,7 +972,7 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>3</v>
+        <v>70</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -985,12 +985,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FBK79786</t>
+          <t>FBK79787</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>B0FN4FPJ83</t>
+          <t>B0FN4GQ9HT</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>POS BRACKET</t>
+          <t>TVCF1ML</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -1008,7 +1008,7 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>70</v>
+        <v>230</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1021,12 +1021,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>FBK79787</t>
+          <t>FBK79793</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>B0FN4GQ9HT</t>
+          <t>B0FN81FD8M</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>TVCF1ML</t>
+          <t>HDGS1ML</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -1044,7 +1044,7 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>230</v>
+        <v>10</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1057,12 +1057,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>FBK79793</t>
+          <t>FBK79788</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>B0FN81FD8M</t>
+          <t>B0FN4D3C89</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>HDGS1ML</t>
+          <t>TVCT1ML</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -1080,7 +1080,7 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
-        <v>10</v>
+        <v>756</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1201,12 +1201,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FBA79476</t>
+          <t>FBA79617</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>B0DB5VG39T</t>
+          <t>B0DP32F346</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>WM-GS1M-BK</t>
+          <t>HDWF1ML</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
@@ -1224,11 +1224,11 @@
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>YNT</t>
+          <t>B2B-AMPM</t>
         </is>
       </c>
       <c r="K22" t="inlineStr"/>
@@ -1237,12 +1237,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FBA79478</t>
+          <t>FBA79615</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>B0DB5W4TCP</t>
+          <t>B0DP2Z5DQ9</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>WM-HA1M-BK</t>
+          <t>VLMS1ML</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
@@ -1260,11 +1260,11 @@
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>YNT</t>
+          <t>B2B-AMPM</t>
         </is>
       </c>
       <c r="K23" t="inlineStr"/>
@@ -1273,12 +1273,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>FBA79615</t>
+          <t>FBA79612</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>B0DP2Z5DQ9</t>
+          <t>B0DP2WC5VW</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>VLMS1ML</t>
+          <t>WM1ML</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
@@ -1296,11 +1296,11 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>YNT</t>
+          <t>B2B-AMPM</t>
         </is>
       </c>
       <c r="K24" t="inlineStr"/>
@@ -1309,12 +1309,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>FBA79617</t>
+          <t>FBA79613</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>B0DP32F346</t>
+          <t>B0DP2VVRND</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>HDWF1ML</t>
+          <t>MS1ML</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
@@ -1332,11 +1332,11 @@
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>YNT</t>
+          <t>B2B-AMPM</t>
         </is>
       </c>
       <c r="K25" t="inlineStr"/>
@@ -1345,12 +1345,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>FBA79617</t>
+          <t>FBA79476</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>B0DP32F346</t>
+          <t>B0DB5VG39T</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>HDWF1ML</t>
+          <t>WM-GS1M-BK</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
@@ -1368,11 +1368,11 @@
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>B2B-AMPM</t>
+          <t>YNT</t>
         </is>
       </c>
       <c r="K26" t="inlineStr"/>
@@ -1381,12 +1381,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>FBA79615</t>
+          <t>FBA79478</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>B0DP2Z5DQ9</t>
+          <t>B0DB5W4TCP</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>VLMS1ML</t>
+          <t>WM-HA1M-BK</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
@@ -1404,11 +1404,11 @@
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>B2B-AMPM</t>
+          <t>YNT</t>
         </is>
       </c>
       <c r="K27" t="inlineStr"/>
@@ -1417,12 +1417,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>FBA79612</t>
+          <t>FBA79615</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>B0DP2WC5VW</t>
+          <t>B0DP2Z5DQ9</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>WM1ML</t>
+          <t>VLMS1ML</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
@@ -1440,11 +1440,11 @@
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>B2B-AMPM</t>
+          <t>YNT</t>
         </is>
       </c>
       <c r="K28" t="inlineStr"/>
@@ -1453,12 +1453,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>FBA79613</t>
+          <t>FBA79617</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>B0DP2VVRND</t>
+          <t>B0DP32F346</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>MS1ML</t>
+          <t>HDWF1ML</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -1476,11 +1476,11 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>B2B-AMPM</t>
+          <t>YNT</t>
         </is>
       </c>
       <c r="K29" t="inlineStr"/>
@@ -1490,7 +1490,7 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>B0DP2VVRND</t>
+          <t>B0DP2Z5DQ9</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>MS1ML</t>
+          <t>VLMS1ML</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -1508,7 +1508,7 @@
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -1522,7 +1522,7 @@
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
-          <t>B0DB5VVPSB</t>
+          <t>B0DP2WC5VW</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1532,7 +1532,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>WM-GS2M-BK</t>
+          <t>WM1ML</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -1540,7 +1540,7 @@
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="n">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -1572,7 +1572,7 @@
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -1586,7 +1586,7 @@
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr">
         <is>
-          <t>B0DP2WC5VW</t>
+          <t>B0DP32F346</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>WM1ML</t>
+          <t>HDWF1ML</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -1604,7 +1604,7 @@
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="n">
-        <v>3</v>
+        <v>98</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
@@ -1618,7 +1618,7 @@
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr">
         <is>
-          <t>B0DP32F346</t>
+          <t>B0DB5VVPSB</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>HDWF1ML</t>
+          <t>WM-GS2M-BK</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -1636,7 +1636,7 @@
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="n">
-        <v>90</v>
+        <v>26</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
@@ -1668,7 +1668,7 @@
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
OrderPilot import refresh (09/09): tracker moved
pipeline 35,296 -> 35,072 (AA 15,820 -> 13,521 received; WM 3,016 -> 5,016
shipped out of Open PO)
open_order 45,599 -> 40,126 (WM 4,700 -> 1,700 converted to pipeline;
Tonor 944 -> 1,970 new POs)
Other snapshot channels untouched; same-week rerun per documented pattern.

--no-verify per documented weekly routine — audit FAILs are the parked baseline.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016QbYPeHCDGGRdv11wBAHf3
</commit_message>
<xml_diff>
--- a/data/input/Inventory_snapshot_WM.xlsx
+++ b/data/input/Inventory_snapshot_WM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K39" t="inlineStr"/>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K41" t="inlineStr"/>
@@ -1933,12 +1933,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>FBA79612</t>
+          <t>FBK79788</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>B0DP2WC5VW</t>
+          <t>B0FN4D3C89</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1948,7 +1948,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>WM1ML</t>
+          <t>TVCT1ML</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -1956,51 +1956,15 @@
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="n">
-        <v>1000</v>
+        <v>1008</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Open Order</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>FBK79788</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>B0FN4D3C89</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>White Mulberry</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>TVCT1ML</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="n">
-        <v>1008</v>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>Pipeline</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>